<commit_message>
Add retry guidance to workbook
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اطلاعات نوآموزان" sheetId="1" r:id="Re952b6ed27424538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنمای ورود" sheetId="2" r:id="Rb054eae1f54241db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اطلاعات نوآموزان" sheetId="1" r:id="R6d0b80e304704102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنمای ورود" sheetId="2" r:id="R1ed4555a52084f43"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -216,7 +216,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -335,6 +335,9 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1574,6 +1577,20 @@
         <x:v>فایلِ تکمیل‌شده حاوی اطلاعات واقعی را در GitHub یا فضای عمومی بارگذاری نکنید.</x:v>
       </x:c>
     </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="41" t="str">
+        <x:v>پس از اصلاح اطلاعات</x:v>
+      </x:c>
+      <x:c r="B44" s="41"/>
+    </x:row>
+    <x:row r="45" ht="50" customHeight="1">
+      <x:c r="A45" s="56" t="str">
+        <x:v>تلاش مجدد</x:v>
+      </x:c>
+      <x:c r="B45" s="53" t="str">
+        <x:v>اگر اطلاعات یک ردیف را اصلاح کردید و می‌خواهید ربات دوباره آن را اجرا کند، وضعیت ربات را دقیقاً به «در انتظار تلاش مجدد» تغییر دهید، فایل را ذخیره و ببندید و سپس ربات را اجرا کنید.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>